<commit_message>
Reestructuración de la web y agregado de Mesa Dulce
</commit_message>
<xml_diff>
--- a/public/data/productos.xlsx
+++ b/public/data/productos.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="92">
   <si>
     <t xml:space="preserve">Nombre</t>
   </si>
@@ -247,109 +247,55 @@
     <t xml:space="preserve">2 bizcochos de vainilla de 14 cm, 1 relleno de crema de dulce de leche. Rinde de 4 a 6 porciones.</t>
   </si>
   <si>
-    <t xml:space="preserve">Pelotita</t>
-  </si>
-  <si>
-    <t xml:space="preserve">regalo4.avif</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Regalos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pelotita de goma multicolor, flexible y resistente, perfecta para juegos, piñatas y souvenirs.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Globos dorados x10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cotillon3.avif</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cotillon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pack de 10 globos dorados de 12", perfectos para decorar fiestas, cumpleaños y eventos especiales.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vela dorada c/ número</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cotillon2.avif</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vela dorada con número, perfecta para decorar tortas de cumpleaños y celebrar cualquier edad.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Globos dorados x20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cotillon1.avif</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pack de 20 globos dorados de 12", perfectos para decorar fiestas, cumpleaños y eventos especiales.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bloques construcción</t>
-  </si>
-  <si>
-    <t xml:space="preserve">regalo5.avif</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Set de bloques de construcción de más de 15 piezas, ideal para crear, jugar y desarrollar la creatividad.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cubo mágico 5 cm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">regalo6.avif</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cubo mágico de colores, perfecto para ejercitar la mente y disfrutar de un desafío entretenido.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Burbujeros Labubu x3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">regalo8.avif</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3 burbujeros con diseño tipo Labubu, perfecto para cumpleaños, cotillón, piñatas y diversión al aire libre.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Burbujeros astro x3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">regalo9.avif</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3 burbujeros con diseño tipo astronauta, perfecto para cumpleaños, cotillón, piñatas y diversión al aire libre.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Burbujeros conejito x3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">regalo7.avif</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3 burbujeros con diseño tipo conejito, perfecto para cumpleaños, cotillón, piñatas y diversión al aire libre.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Platos desechables</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cotillon4.avif</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10 platos desechables que son resistentes e ideales para servir porciones de torta de forma práctica e higiénica.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vasos desechables</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cotillon5.avif</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10 vasos desechables resistentes, ideales para bebidas en fiestas y celebraciones.</t>
+    <t xml:space="preserve">Cake pops x 12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mesadulce1.avif</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MesaDulce</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bizcocho suave, baño de chocolate y decoración a mano. Se venden por docena. Ideales para regalos y eventos. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Muffins x 12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mesadulce2.avif</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Esponjosos, húmedos y recién horneados. Se venden por docena. Ideales para el desayuno, la merienda y regalos. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paletas x 12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mesadulce3.avif</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chocolate de calidad en su palito, con decoración a mano. Se venden por docena. Ideales para regalos y eventos. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Promo 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">promos1.avif</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Promos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Torta personalizada de 10 porciones + 12 postres de su elección</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Promo 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">promos2.avif</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Torta personalizada de 20 porciones + 12 postres de su elección</t>
   </si>
 </sst>
 </file>
@@ -574,13 +520,13 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="25.04"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="5.98"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="11.82"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="8.9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="14.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="10.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="106"/>
   </cols>
   <sheetData>
@@ -997,7 +943,7 @@
         <v>75</v>
       </c>
       <c r="B25" s="1" t="n">
-        <v>35</v>
+        <v>900</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>76</v>
@@ -1014,49 +960,49 @@
         <v>79</v>
       </c>
       <c r="B26" s="1" t="n">
-        <v>120</v>
+        <v>900</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>80</v>
       </c>
       <c r="D26" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="E26" s="3" t="s">
         <v>81</v>
-      </c>
-      <c r="E26" s="3" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B27" s="1" t="n">
+        <v>900</v>
+      </c>
+      <c r="C27" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="B27" s="1" t="n">
-        <v>90</v>
-      </c>
-      <c r="C27" s="1" t="s">
+      <c r="D27" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="E27" s="3" t="s">
         <v>84</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="E27" s="3" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B28" s="1" t="n">
+        <v>2400</v>
+      </c>
+      <c r="C28" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="B28" s="1" t="n">
-        <v>220</v>
-      </c>
-      <c r="C28" s="1" t="s">
+      <c r="D28" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="D28" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="E28" s="3" t="s">
+      <c r="E28" s="1" t="s">
         <v>88</v>
       </c>
     </row>
@@ -1065,118 +1011,16 @@
         <v>89</v>
       </c>
       <c r="B29" s="1" t="n">
-        <v>60</v>
+        <v>3200</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>90</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="E29" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="E29" s="1" t="s">
         <v>91</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="B30" s="1" t="n">
-        <v>70</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="E30" s="3" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="B31" s="1" t="n">
-        <v>135</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="E31" s="3" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="B32" s="1" t="n">
-        <v>125</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="D32" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="E32" s="3" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="B33" s="1" t="n">
-        <v>130</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="E33" s="3" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="B34" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="D34" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="E34" s="3" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="B35" s="1" t="n">
-        <v>120</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="D35" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="E35" s="3" t="s">
-        <v>109</v>
       </c>
     </row>
   </sheetData>

</xml_diff>